<commit_message>
Auto: 2026-09-27 scrape results
</commit_message>
<xml_diff>
--- a/results/scraped_Cape_Town_Community_Development.xlsx
+++ b/results/scraped_Cape_Town_Community_Development.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="113">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -40,58 +40,64 @@
     <t>Source</t>
   </si>
   <si>
-    <t>edrelectronics.com</t>
-  </si>
-  <si>
-    <t>Blog</t>
-  </si>
-  <si>
-    <t>Service Area | EDR Electronics | Arlington Heights,IL</t>
-  </si>
-  <si>
-    <t>FAQ -edrelectronics.com</t>
-  </si>
-  <si>
-    <t>edrelectronics</t>
-  </si>
-  <si>
-    <t>Geo Pages -edrelectronics.com</t>
-  </si>
-  <si>
-    <t>Machinery Repair Services for Industrial | EDR Electronics Inc.</t>
-  </si>
-  <si>
-    <t>Automation Control Services | EDR Electronics | Arlington Heights,IL</t>
-  </si>
-  <si>
-    <t>#1Best JDM Imports In Colorado- JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>JDM Sport Classics - Classic Japanese Car Importers</t>
-  </si>
-  <si>
-    <t>2000 HondaCivicG - JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>Hondacivic-ferio 1993 - JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>Toyota Supra inColorado- JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>#1Best JDM Imports In North Carolina- JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>Nissan Skyline in Colorado- JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>#1Best JDM Imports In New Jersey- JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>#1Best JDM Imports In Illinois- JDM Sport Classics</t>
-  </si>
-  <si>
-    <t>#1Best JDM Imports In Mississippi- JDM Sport Classics</t>
+    <t>community（英语单词）_百度百科</t>
+  </si>
+  <si>
+    <t>Community-Wikipedia</t>
+  </si>
+  <si>
+    <t>COMMUNITY中文 (简体)翻译：剑桥词典</t>
+  </si>
+  <si>
+    <t>community是什么意思_community的翻译_音标_读音_用法_例句_爱词 …</t>
+  </si>
+  <si>
+    <t>COMMUNITY| English meaning - Cambridge Dictionary</t>
+  </si>
+  <si>
+    <t>COMMUNITYDefinition &amp; Meaning -Merriam-Webster</t>
+  </si>
+  <si>
+    <t>浅谈词汇多重意义之三："community" 未必是“社区” - 知乎</t>
+  </si>
+  <si>
+    <t>COMMUNITY释义 | 柯林斯英语词典</t>
+  </si>
+  <si>
+    <t>Community (TV series) -Wikipedia</t>
+  </si>
+  <si>
+    <t>community- 搜索 词典</t>
+  </si>
+  <si>
+    <t>Honda CivicFamily: Models &amp; Price | Honda</t>
+  </si>
+  <si>
+    <t>Honda Civic- Wikipedia</t>
+  </si>
+  <si>
+    <t>2026CivicSedan - Fun &amp; Sporty Compact w/ Hybrid Option</t>
+  </si>
+  <si>
+    <t>Used HondaCivicfor Sale inEscondido,CA- Autotrader</t>
+  </si>
+  <si>
+    <t>New HondaCivicfor Sale inEscondido,CA</t>
+  </si>
+  <si>
+    <t>New and Used Honda DealerEscondido CA- Honda ofEscondido</t>
+  </si>
+  <si>
+    <t>New HondaCivicfor Sale inEscondido,CA- Autotrader</t>
+  </si>
+  <si>
+    <t>2026Honda CivicReview, Pricing, and Specs - Car and Driver</t>
+  </si>
+  <si>
+    <t>Used HondaCivicnearEscondido,CAfor sale - CarMax</t>
+  </si>
+  <si>
+    <t>2026Honda CivicPrice, Reviews, Pictures &amp; More | Kelley Blue Book</t>
   </si>
   <si>
     <t>Nextdoor</t>
@@ -103,85 +109,85 @@
     <t>Join your neighborhood |Nextdoor</t>
   </si>
   <si>
+    <t>Nextdoor - Discover yourneighbourhood</t>
+  </si>
+  <si>
+    <t>Login - Nextdoor</t>
+  </si>
+  <si>
+    <t>The Neighbourhood-Wikipedia</t>
+  </si>
+  <si>
+    <t>The Neighbourhood-YouTube</t>
+  </si>
+  <si>
+    <t>TheNeighbourhood– Official Biography, Songs, Albums &amp; Tour Dates</t>
+  </si>
+  <si>
     <t>TheNeighbourhood- Wourld Tour</t>
   </si>
   <si>
-    <t>The Neighbourhood-Wikipedia</t>
-  </si>
-  <si>
-    <t>The Neighbourhood-YouTube</t>
-  </si>
-  <si>
-    <t>Nextdoor - Discover yourneighbourhood</t>
-  </si>
-  <si>
     <t>TheNeighbourhood- Sweater Weather (Official Video)</t>
   </si>
   <si>
-    <t>Neighbourhood| Definition &amp; Facts | Britannica</t>
-  </si>
-  <si>
-    <t>TheNeighbourhood– Official Biography, Songs, Albums &amp; Tour Dates</t>
+    <t>Residence vs.Residents: What's the Difference? - Grammarly</t>
   </si>
   <si>
     <t>The Residents Official Site</t>
   </si>
   <si>
-    <t>Residence vs.Residents: What's the Difference? - Grammarly</t>
-  </si>
-  <si>
     <t>The Residents-Wikipedia</t>
   </si>
   <si>
-    <t>MichiganResidentsDatabase Search</t>
-  </si>
-  <si>
     <t>RESIDENTDefinition &amp; Meaning -Merriam-Webster</t>
   </si>
   <si>
+    <t>Residents– COUNTY OF LOS ANGELES</t>
+  </si>
+  <si>
+    <t>RESIDENT| English meaning - Cambridge Dictionary</t>
+  </si>
+  <si>
+    <t>RESIDENT| definition in the Cambridge English Dictionary</t>
+  </si>
+  <si>
+    <t>RESIDENTSDefinition &amp; Meaning | Dictionary.com</t>
+  </si>
+  <si>
     <t>Live &amp; Preserved - TheResidents</t>
   </si>
   <si>
-    <t>RESIDENT| definition in the Cambridge English Dictionary</t>
-  </si>
-  <si>
-    <t>RESIDENT| English meaning - Cambridge Dictionary</t>
-  </si>
-  <si>
-    <t>RESIDENTSDefinition &amp; Meaning | Dictionary.com</t>
-  </si>
-  <si>
-    <t>The Residents - Topic-YouTube</t>
-  </si>
-  <si>
-    <t>WardTransport &amp; Logistics | LTL Freight Services</t>
-  </si>
-  <si>
-    <t>WARDDefinition &amp; Meaning -Merriam-Webster</t>
-  </si>
-  <si>
-    <t>Ward-Wikipedia</t>
-  </si>
-  <si>
-    <t>WARD| English meaning - Cambridge Dictionary</t>
-  </si>
-  <si>
-    <t>WardApp - Apps on Google Play</t>
-  </si>
-  <si>
-    <t>Montgomery Ward|Buy Now Pay LaterCredit</t>
-  </si>
-  <si>
-    <t>What is aWard? The 'Bridgerton' Term Explained - Parade</t>
-  </si>
-  <si>
-    <t>Ward- Definition, Meaning &amp; Synonyms | Vocabulary.com</t>
-  </si>
-  <si>
-    <t>Ward (United States) -Wikipedia</t>
-  </si>
-  <si>
-    <t>WARDDefinition &amp; Meaning |Dictionary.com</t>
+    <t>Residents- definition ofresidentsby The Free Dictionary</t>
+  </si>
+  <si>
+    <t>Scores &amp; Fixtures - Football - BBC Sport</t>
+  </si>
+  <si>
+    <t>Football - latest news today, results &amp; video highlights - BBC Sport</t>
+  </si>
+  <si>
+    <t>Premier League - Scores &amp; Fixtures - Football - BBC Sport</t>
+  </si>
+  <si>
+    <t>Championship - Scores &amp; Fixtures - Football - BBC Sport</t>
+  </si>
+  <si>
+    <t>Premier League Football - Latest news, results, stats &amp; transfers - BBC</t>
+  </si>
+  <si>
+    <t>Rugby Union - latest news today, results &amp; video - BBC Sport</t>
+  </si>
+  <si>
+    <t>Cricket – Ashes, Test, T20 &amp; ODI news, scores &amp; results - BBC</t>
+  </si>
+  <si>
+    <t>Scottish Premiership - Scores &amp; Fixtures - Football - BBC Sport</t>
+  </si>
+  <si>
+    <t>Irish - Scores &amp; Fixtures - Football - BBC Sport</t>
+  </si>
+  <si>
+    <t>England - Scores &amp; Fixtures - Football - BBC Sport</t>
   </si>
   <si>
     <t>Community Development</t>
@@ -190,151 +196,160 @@
     <t>Cape Town</t>
   </si>
   <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=3a80764835c2913f122478e66d337a550cb51b5c4bc1c292baafec8fd5a2d3c8JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly9lZHJlbGVjdHJvbmljcy5jb20vaW5kZXguaHRtbA&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=ef2e27d229c94b48a822ddf2638413085b0500d8fc0dbfab554582033940b81fJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly93d3cuZWRyZWxlY3Ryb25pY3MuY29tL2Jsb2c&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=e0f7d7fef60edac61ceae4031eb814af2b5f0fab296634b32d37c2669c02d034JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly93d3cuZWRyZWxlY3Ryb25pY3MuY29tL3NlcnZpY2UtYXJlYQ&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=21891dc04330ab815b583bc009e70d2e7e530de586ef4ebaa1a3551691105d22JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly93d3cuZWRyZWxlY3Ryb25pY3MuY29tL2ZhcQ&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=ed62d5684685564a5d6a8676fc6fff69265c2258a9d8368321fdbb4e056c9c72JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly93d3cuZWRyZWxlY3Ryb25pY3MuY29tL2ZlZWQvcnNzMg&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=bf4c0065bd52ad4a678d0b3c51c0e4b1f076119b7ecc05d60bd586bbd13a1ea8JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly93d3cuZWRyZWxlY3Ryb25pY3MuY29tL2dlby1wYWdlcy9lbGstZ3JvdmUtdmlsbGFnZS1pbA&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=81a53e4e5e87390812cbb96d966a92d2412c5b72488473f14fecfebc4cd44881JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly93d3cuZWRyZWxlY3Ryb25pY3MuY29tL21hY2hpbmVyeS1yZXBhaXItc2VydmljZXMtZm9yLWluZHVzdHJpYWwtZXF1aXBtZW50LWluLWVsay1ncm92ZS12aWxsYWdlLWls&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=08854ba8e0f85a1022558edd60c0d7ca81185bd1101bf3b5c0fd77ced80953d6JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=273716c9-1226-6f58-03d0-012813ce6e71&amp;u=a1aHR0cHM6Ly93d3cuZWRyZWxlY3Ryb25pY3MuY29tL2NvbnRhY3Q&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=ee5b444ef3f84945ee2b53885cfd874ca47ef9b7e33dc6f5f0cd0282807ca935JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS8xLWJlc3QtamRtLWltcG9ydHMtaW4tY29sb3JhZG8v&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=0f5edac4396fd04858d978869638c47fb13c090afce9bf76396f8cc579790c39JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS8&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=2d88e28b713d3398845e106d86719f4780a0908fde114a890c59a0d40155b3f1JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS9pbnZlbnRvcnkvMjAwMC1ob25kYS1jaXZpYy1nLw&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=a24593764d9192357c329f1f3e4720c6a75deeba8d1e9edd5c230ae3ce7f3c88JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS9pbnZlbnRvcnkvMTk5My1ob25kYS1jaXZpYy1mZXJpby8&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=98185868bba99d95886dd98e59994ed070c1ac59ccc663720e6c5e1a397e01e8JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS90b3lvdGEtc3VwcmEtaW4tY29sb3JhZG8v&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=2e36502a8b5a32df8de67808a201124ed1c2aec91ff56c605334ada9a55d1469JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS8xLWJlc3QtamRtLWltcG9ydHMtaW4tbm9ydGgtY2Fyb2xpbmEv&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=776321657aad829e4b515bb9fd51039ccead1384297490f73e32fb2295e5f1d3JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS9uaXNzYW4tc2t5bGluZS1pbi1jb2xvcmFkby8&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=c17fa6d741386ea800a879827f5c6974fbff98c4097ae19c27346f1daf0b0677JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS8xLWJlc3QtamRtLWltcG9ydHMtaW4tbmV3LWplcnNleS8&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=f69553c22fc96ab3ca1e45099e564cf1b3f16768ff7743261214dfdbfa810ed3JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS8xLWJlc3QtamRtLWltcG9ydHMtaW4taWxsaW5vaXMv&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=06ba0039c47e65f0554e4dbd5d82f06b49f9fdf5ed5119c753cf7dd9016b8301JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=156bb91c-62bf-6f92-3b0c-aefd634e6e65&amp;u=a1aHR0cHM6Ly9qZG1zcG9ydGNsYXNzaWNzLmNvbS8xLWJlc3QtamRtLWltcG9ydHMtaW4tbWlzc2lzc2lwcGkv&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=4b1ff4c60df77f9310998386cbcca48454d3f51a818b92c843897c64c1d44967JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly9uZXh0ZG9vci5jb20v&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=907d81ad4cee089d0df8e4ba2a247abae2a8c6f65fb407e3809b4f68ae3ea2f6JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly9lbi5tLndpa2lwZWRpYS5vcmcvd2lraS9OZWlnaGJvdXJob29k&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=aad225ccf3a977a4a4a49a5f672b6dbbea7f3fcd6b2e0658617384321630f752JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly9uZXh0ZG9vci5jb20vZmluZC1uZWlnaGJvcmhvb2Qv&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=3164930fe065ef6bd521e0d950a446ae5dbc5cb7b4fb6ff734bfc4ad720b6597JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly90b3VyLnRoZW5iaGQuY29tLw&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=d1a8c5afc3c53c722ac16797bf00e95f2a18020353bd137f50714ea1046a462eJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly9lbi5tLndpa2lwZWRpYS5vcmcvd2lraS9UaGVfTmVpZ2hib3VyaG9vZA&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=f75f2675f77e57abafeed8aefb5d576a8f08616e8ec1c97b674ab2fc7b7f9ae5JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly93d3cueW91dHViZS5jb20vY2hhbm5lbC9VQ0RBWHVzWXdSSnBpU1AyQ0huWG5Wbnc&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=09868152caa84d4891feff222f7d00f846d4b18bba812f62891a2ce2995638f9JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly9jYS5uZXh0ZG9vci5jb20v&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=c7068c72fdda7b544eecdda3304d894a01e8bf035bdbd8e60858a576652170d8JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly9tLnlvdXR1YmUuY29tL3dhdGNoP3Y9R0Nkd0toVHROTnc&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=885dab08350327586faa09e9fb3ccbd0ed6cc92691baec353a5d405b5f42797cJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly93d3cuYnJpdGFubmljYS5jb20vdG9waWMvbmVpZ2hib3Job29kLXNvY2lvbG9neQ&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=8213fd9ecd1e7641779cd413c98ab1404b8f8b43efd98d80bd598178eb36c5e8JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=12ad742a-fe33-6373-1f29-63cbffa462f5&amp;u=a1aHR0cHM6Ly93d3cudGhlbmVpZ2hib3VyaG9vZC5uZXQvYmlv&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=f805389ab91dd3498d7d560c2611e7488e45d5f65b25bc1320cfcfe463e7ca0fJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly93d3cucmVzaWRlbnRzLmNvbS8&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=815aea4f9950789035acde2214d81768f024366a6ceae69dad58d9f1af89ad9fJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly93d3cuZ3JhbW1hcmx5LmNvbS9jb21tb25seS1jb25mdXNlZC13b3Jkcy9yZXNpZGVuY2UtdnMtcmVzaWRlbnRzP21zb2NraWQ9Mjc3NTQ0NTg3YzgxNmJhODBmY2Y1M2I5N2Q5OTZhOTQ&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=dc129713bd63e13d3c801a47033a69bb0c69431dfd262f3a76b59dde3f4ed7a2JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly9lbi53aWtpcGVkaWEub3JnL3dpa2kvVGhlX1Jlc2lkZW50cw&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=8cb5a97a25d3e5e2d60cb902c5ab4133be547b3c6ee488a267a29ce542868121JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly93d3cubWljaGlnYW5yZXNpZGVudGRhdGFiYXNlLmNvbS8&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=5eb45a5c9de12189cfffca26da64e6b62d68482961c597ed05d3e88172ca9ed1JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly93d3cubWVycmlhbS13ZWJzdGVyLmNvbS9kaWN0aW9uYXJ5L3Jlc2lkZW50&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=f0f9e7e4328bf730c6eacb012449099e5d27e3b096f6a047beecc775f7102441JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly93d3cucmVzaWRlbnRzLmNvbS90b3VyZGF0ZXMv&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=3f491feaca0bec746cb0abde0d99550479ae2be20f7cfe9faf659b8a4f72e63fJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly9kaWN0aW9uYXJ5LmNhbWJyaWRnZS5vcmcvdXMvZGljdGlvbmFyeS9lbmdsaXNoL3Jlc2lkZW50&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=e1cf4232ba900f88ded248a67dd1c29dbb7a1921b9f4a5aad18bc8bebf601925JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly9kaWN0aW9uYXJ5LmNhbWJyaWRnZS5vcmcvZGljdGlvbmFyeS9lbmdsaXNoL3Jlc2lkZW50&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=c0f53a264a0467ed8a96d1320b6c26b82231219ee4318b598d415b629ca31c49JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly93d3cuZGljdGlvbmFyeS5jb20vYnJvd3NlL3Jlc2lkZW50cw&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=c3bc3847f5c86ed3b81041b460d59b80fce530d43c9873e819a14da1977d3097JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=27754458-7c81-6ba8-0fcf-53b97d996a94&amp;u=a1aHR0cHM6Ly93d3cueW91dHViZS5jb20vY2hhbm5lbC9VQ3IyeGRUWXJZLVEwMlBWZWJyVGRnaVE&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=9c37bbce9b70834f43cf69109b08da15895b86960cea42c9210dd4d2052c18ecJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly93d3cud2FyZHRsYy5jb20v&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=c28f9501890c507a4551afe6e5dd647ab052c9a7f7cdd4481c14da8f9cd53727JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly93d3cubWVycmlhbS13ZWJzdGVyLmNvbS9kaWN0aW9uYXJ5L3dhcmQ&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=c8359c3216ecc23fbf3b663fac73db77a56d364f56cf064cc7e4a316e3d08f95JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly9lbi53aWtpcGVkaWEub3JnL3dpa2kvV2FyZA&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=9ff8840ec89911c67215c08e7174809869279fa8e160446014f217b7b1d58f7cJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly9kaWN0aW9uYXJ5LmNhbWJyaWRnZS5vcmcvZGljdGlvbmFyeS9lbmdsaXNoL3dhcmQ&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=7d5f35ab28a719ef6ab8b77006d5663f95384e679bc437dd98d19e3d9ea804bfJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly9wbGF5Lmdvb2dsZS5jb20vc3RvcmUvYXBwcy9kZXRhaWxzP2lkPWNvbS50ZWNocmNzLndhcmRhcHAmaGw9ZW4tVVM&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=1c17ea43c0f9ab4c113bb76cb7c9b0657f50953a5f740cdd73bf5d8af5803475JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly93d3cud2FyZHMuY29tLz9tc29ja2lkPTIwNTgxNTZhNjhmYjZiNjcyMzZmMDI4YjY5NTg2YTY0&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=7e49ff612e6519f0543e6d90b375b046a5adee99474b2d2b0062c6224a0f6b06JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly9wYXJhZGUuY29tL3R2L3doYXQtaXMtYS13YXJkLXRoZS1icmlkZ2VydG9uLXRlcm0tZXhwbGFpbmVk&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=cf9cc1b19588f72ddfb92ce38d7b51aacea1648fcff866a30bfe721fc2c8833eJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly93d3cudm9jYWJ1bGFyeS5jb20vZGljdGlvbmFyeS93YXJk&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=34a6d32ad98f220bbac724f5d62d323cdf26f1be46cd29d2b12752f2ab6c1f47JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly9lbi53aWtpcGVkaWEub3JnL3dpa2kvV2FyZF8oVW5pdGVkX1N0YXRlcyk&amp;ntb=1</t>
-  </si>
-  <si>
-    <t>https://www.bing.com/ck/a?!&amp;&amp;p=414ae16748f1f07d0c8733269d0663e755c5aea6f74f3a134ad2b74b87d8d6daJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2058156a-68fb-6b67-236f-028b69586a64&amp;u=a1aHR0cHM6Ly93d3cuZGljdGlvbmFyeS5jb20vYnJvd3NlL3dhcmQ&amp;ntb=1</t>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=07c5e372adef6f4922049baed7860050b9ab6c4871da10ffaee8969c61af40d7JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly9iYWlrZS5iYWlkdS5jb20vaXRlbS9jb21tdW5pdHkvOTM3MjM0OQ&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=530e019fcd98e2eb4640c81aced86158b5f2c02be8f16e038b1a284edbfb4f57JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly9lbi5tLndpa2lwZWRpYS5vcmcvd2lraS9Db21tdW5pdHk&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=e1fca2f37d1c0dd32c549bdcaf55093070465f9e268602c47bfdc43e4e87e3e0JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly9kaWN0aW9uYXJ5LmNhbWJyaWRnZS5vcmcvemhzLyVFOCVBRiU4RCVFNSU4NSVCOC8lRTglOEIlQjElRTglQUYlQUQtJUU2JUIxJTg5JUU4JUFGJUFELSVFNyVBRSU4MCVFNCVCRCU5My9jb21tdW5pdHk&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=aafcebdeb81fbcb407d1d780729234220180c5d5d0120e49902df411fef71c1cJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly93d3cuaWNpYmEuY29tL3dvcmQ_dz1jb21tdW5pdHk&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=be33d9958b6fc40eb099f120696b12b40793260489b03047fa3ee7b398b6dc24JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly9kaWN0aW9uYXJ5LmNhbWJyaWRnZS5vcmcvZGljdGlvbmFyeS9lbmdsaXNoL2NvbW11bml0eQ&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=767849f19f0a4a085ddd9810707df55a2bc73862ed4e3e1fae47d87b5df2dd64JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly93d3cubWVycmlhbS13ZWJzdGVyLmNvbS9kaWN0aW9uYXJ5L2NvbW11bml0eQ&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=716ea6e472ed86e9538089d155eb173b383e83eee5e09c937088fce311c924a6JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly96aHVhbmxhbi56aGlodS5jb20vcC80MDIxODA0MTE&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=7db61797e5da9c48c4f6a327467ceae92f1e9878f5f00834233f35d32f3c07b3JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly93d3cuY29sbGluc2RpY3Rpb25hcnkuY29tL3poL2RpY3Rpb25hcnkvZW5nbGlzaC9jb21tdW5pdHk&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=f7d6566ce5f2efeb753643196cf370d07b0082d88f5a237548a020a773d5b0adJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly9lbi5tLndpa2lwZWRpYS5vcmcvd2lraS9Db21tdW5pdHlfKFRWX3Nlcmllcyk&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=702ff853837d75916580a1a336a781206e90e2b31db5a870c637fac297222955JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=0fee8536-9213-6d6a-39f9-92d793d76c55&amp;u=a1aHR0cHM6Ly9nbG9iYWwuYmluZy5jb20vZGljdC9zZWFyY2g_cT1jb21tdW5pdHkmRk9STT1CRFZTUDYmY2M9Y24&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=45f98c2cecdfc9fe82b125745a639fda063749b1b4738411418a3c45003260e7JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly9hdXRvbW9iaWxlcy5ob25kYS5jb20vY2l2aWM&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=459a2320c4868aee44c02e6c816fe01de0601da82e1e4acf05036a788c4d0f4dJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly9lbi5tLndpa2lwZWRpYS5vcmcvd2lraS9Ib25kYV9DaXZpYw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=0acf22f5d0a9edd8f4f0fed29073cfbc039d13fdbd55d39dc9a433d3c66499edJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly9hdXRvbW9iaWxlcy5ob25kYS5jb20vY2l2aWMtc2VkYW4&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=6d03d4c26ab01e3730aa8736b94d84bc1d54dc4a7761778d1ddd3abe2671a691JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly93d3cuYXV0b3RyYWRlci5jb20vY2Fycy1mb3Itc2FsZS9ob25kYS9jaXZpYy9lc2NvbmRpZG8tY2E_bXNvY2tpZD0xZTYwNmRmMjM1MmU2MzAzMDYzYjdhMTMzNGQxNjIxMQ&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=75e8b44677e604ae567afe4cbbdeee807b4be1478648512bdc906ab95a78935aJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly93d3cuaG9uZGFvZmVzY29uZGlkby5jb20vbmV3LXZlaGljbGVzL2NpdmljLXNlZGFuLw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=e4b5e7a91539f6e8a9070fb3eb9897ab4009845c80f34dffa48d1942563d0644JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly93d3cuaG9uZGFvZmVzY29uZGlkby5jb20v&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=a0db2b7a342fa15a5bb7ebedab4332043d1c8a35735b1c73da576b418d7cc1a5JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly93d3cuYXV0b3RyYWRlci5jb20vY2Fycy1mb3Itc2FsZS9uZXctY2Fycy9ob25kYS9jaXZpYy9lc2NvbmRpZG8tY2E_bXNvY2tpZD0xZTYwNmRmMjM1MmU2MzAzMDYzYjdhMTMzNGQxNjIxMQ&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=8010d1112fd85216c7577af4ed6c620ad37ba82b877b087f00e6550f7e454f26JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly93d3cuY2FyYW5kZHJpdmVyLmNvbS9ob25kYS9jaXZpYw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=7a288e7851bcaf1694fd4dc48625a4dd38ba3d960b4fb52b9b95c6ef362c6fceJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly93d3cuY2FybWF4LmNvbS9jYXJzL2hvbmRhL2NpdmljP2xvY2F0aW9uPWVzY29uZGlkbytjYSZtc29ja2lkPTFlNjA2ZGYyMzUyZTYzMDMwNjNiN2ExMzM0ZDE2MjEx&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=e928f316fa10db00119f1cd17870c9458a2ab6730ead1cb6bf791ad9401c4b20JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1e606df2-352e-6303-063b-7a1334d16211&amp;u=a1aHR0cHM6Ly93d3cua2JiLmNvbS9ob25kYS9jaXZpYy8_bXNvY2tpZD0xZTYwNmRmMjM1MmU2MzAzMDYzYjdhMTMzNGQxNjIxMQ&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=e57795932479f8b57108726e500fa9c1760c2e8f1243b6042cc362c03dfac659JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly9uZXh0ZG9vci5jb20v&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=2325e62e1e33f561bfd232334e17c5a9ae5209b213fb80e8570389fd31e90f99JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly9lbi53aWtpcGVkaWEub3JnL3dpa2kvTmVpZ2hib3VyaG9vZA&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=11a6530caae8c2f43b01f6b4a0abb1efc4dd3b04dd688e45a7b9aca90cedd1c3JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly9uZXh0ZG9vci5jb20vZmluZC1uZWlnaGJvcmhvb2Qv&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=0f959bdc42a8c9e48350c871ab36c0ab697db017fdd882815a942040dbbade35JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly9jYS5uZXh0ZG9vci5jb20v&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=3904acca6f83214d0ec9484a4d782f127b667d10eeb207510f35621b2a555f0dJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly9jYS5uZXh0ZG9vci5jb20vbG9naW4v&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=2a43d7edf0e08044c3ad961d05a278f81e1da7ae8020552bb4c9e6b96323c949JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly9lbi53aWtpcGVkaWEub3JnL3dpa2kvVGhlX05laWdoYm91cmhvb2Q&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=d73cf733e17bcb7ad784a1ecda0d06b75b622fce90e83e470b40c55e351992eaJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly93d3cueW91dHViZS5jb20vY2hhbm5lbC9VQ0RBWHVzWXdSSnBpU1AyQ0huWG5Wbnc&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=ecee449cb907baccc2552b797be2614c94b7844806b8089492ac1db5704a3f7bJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly93d3cudGhlbmVpZ2hib3VyaG9vZC5uZXQvYmlv&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=dc736d65015dd835b3de9d0151ac79dac621dcd0e06d401bb99a8a1fde2e97f4JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly90b3VyLnRoZW5iaGQuY29tLw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=836616998f4d8e76524355b672375a6164c4b83687e6a228864a152dc0e6295eJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=2e3f9143-6a83-60af-2d91-86a26b246120&amp;u=a1aHR0cHM6Ly93d3cueW91dHViZS5jb20vd2F0Y2g_dj1HQ2R3S2hUdE5Odw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=457dc8c7b17c24b32cd0be6762126c82021b43ccd027be98e49c6bfebdb9b36eJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly93d3cuZ3JhbW1hcmx5LmNvbS9jb21tb25seS1jb25mdXNlZC13b3Jkcy9yZXNpZGVuY2UtdnMtcmVzaWRlbnRzP21zb2NraWQ9MWE3NmY1NWU2ZWMwNjdkMjEyNzhlMmJmNmY5NjY2NjI&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=f8dc2e36d1eab22ee146b6f41eab89b19f60e53f57108d34841ff3bde48cfebaJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly93d3cucmVzaWRlbnRzLmNvbS8&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=19ec86ab9d7b3f1340083a0707854f8eaa2cac8bb92213df3f1d9f84216033baJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly9lbi53aWtpcGVkaWEub3JnL3dpa2kvVGhlX1Jlc2lkZW50cw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=5b5da55df008ac49c290d4ea46169f1e2f0ab8137e59637ecdbca58f740f7a7fJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly93d3cubWVycmlhbS13ZWJzdGVyLmNvbS9kaWN0aW9uYXJ5L3Jlc2lkZW50&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=cb8dca24adb9b0a79d98e2394f5ef59dce3ac9c7835da10633c76e545e15e31aJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly9sYWNvdW50eS5nb3YvcmVzaWRlbnRzLw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=39c37090d1afa7df144c019735e709db69dc41e90889073649defe4fc1c48576JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly9kaWN0aW9uYXJ5LmNhbWJyaWRnZS5vcmcvZGljdGlvbmFyeS9lbmdsaXNoL3Jlc2lkZW50&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=403799c010bb81bb216f380e7c59c5705c1c89e9fcd667b3f4c5c4bde4901164JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly9kaWN0aW9uYXJ5LmNhbWJyaWRnZS5vcmcvdXMvZGljdGlvbmFyeS9lbmdsaXNoL3Jlc2lkZW50&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=2f16d91aed198cca04fd113d2bffd0260fbc955b14494686a51a81b3851f73d0JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly93d3cuZGljdGlvbmFyeS5jb20vYnJvd3NlL3Jlc2lkZW50cw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=ca4df5116d2ddb7b9acc7fceea53a694f60bdb5681fa8358e1294e93aa416395JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly93d3cucmVzaWRlbnRzLmNvbS90b3VyZGF0ZXMv&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=be6ea7ecd02123ea9edd6cf083a61fc8df57dccaf0850b952fe816906e1ec498JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1a76f55e-6ec0-67d2-1278-e2bf6f966662&amp;u=a1aHR0cHM6Ly93d3cudGhlZnJlZWRpY3Rpb25hcnkuY29tL1Jlc2lkZW50cw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=7996d8292a81858a627fc7d5abfcba95639670bce09e6716caf9ff8c4453d40dJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxsL3Njb3Jlcy1maXh0dXJlcw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=dd5a69d180192451fc074d2622cef56da649dc26ca3bf5ba1423515fefe28903JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxs&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=756ffb1f9cf31aa2fff28fa4d84ea5106bf0d9490a2104718fca3af428b7009dJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxsL3ByZW1pZXItbGVhZ3VlL3Njb3Jlcy1maXh0dXJlcw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=9cd165f28a2391b60295a0254b5a00055728a510642a374018d0f04a80dc5fd8JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxsL2NoYW1waW9uc2hpcC9zY29yZXMtZml4dHVyZXM&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=1f6dad3e8461218a7af3c237b0c0b207ce32ae2af17cd47a9526d278314d94ecJmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxsL3ByZW1pZXItbGVhZ3Vl&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=ae56f9d6cbbf9126d3d41b29f1ee42dd603595c637fca1c08a0cefa3b06cb114JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L3J1Z2J5LXVuaW9u&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=e949d802f3ef8cf398c6845a64ec146c1b3911c49a75a9e77e22f7c34a566418JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2NyaWNrZXQ&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=3ef0f1b3ceb4482fddb9b79ee971df3f98796784edf314dd3bed2a1b20066822JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxsL3Njb3R0aXNoLXByZW1pZXJzaGlwL3Njb3Jlcy1maXh0dXJlcw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=44f334d83a24df1e564a5b01e342d480ce48a1bfd0806708133fc14b671c1ab8JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxsL2lyaXNoL3Njb3Jlcy1maXh0dXJlcw&amp;ntb=1</t>
+  </si>
+  <si>
+    <t>https://www.bing.com/ck/a?!&amp;&amp;p=99d5ce89e56a71def639ab660bcd46aaa4bff723f3cc17ff9d6393216c618461JmltdHM9MTc5MDQ2NzIwMA&amp;ptn=3&amp;ver=2&amp;hsh=4&amp;fclid=1dd0d406-b495-6a40-2dd1-c3e7b59a6bb4&amp;u=a1aHR0cHM6Ly93d3cuYmJjLmNvLnVrL3Nwb3J0L2Zvb3RiYWxsL3RlYW1zL2VuZ2xhbmQvc2NvcmVzLWZpeHR1cmVz&amp;ntb=1</t>
   </si>
   <si>
     <t>Cape Town CBD</t>
+  </si>
+  <si>
+    <t>Green Point</t>
   </si>
   <si>
     <t>Bing</t>
@@ -682,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -716,19 +731,19 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -736,19 +751,19 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -756,19 +771,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G4" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H4" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -776,19 +791,19 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H5" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -796,19 +811,19 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -816,19 +831,19 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H7" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -836,19 +851,19 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H8" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -856,19 +871,19 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G9" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H9" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -876,19 +891,19 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -896,19 +911,19 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H11" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -916,19 +931,19 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H12" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -936,19 +951,19 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G13" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -956,19 +971,19 @@
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H14" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -976,19 +991,19 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G15" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H15" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -996,19 +1011,19 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H16" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1016,19 +1031,19 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H17" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1036,19 +1051,19 @@
         <v>24</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G18" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H18" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1056,19 +1071,19 @@
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G19" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H19" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1076,19 +1091,19 @@
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G20" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H20" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1096,19 +1111,19 @@
         <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G21" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H21" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1116,19 +1131,19 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G22" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H22" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1136,19 +1151,19 @@
         <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G23" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H23" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1156,19 +1171,19 @@
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G24" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H24" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1176,19 +1191,19 @@
         <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G25" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H25" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1196,19 +1211,19 @@
         <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G26" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H26" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1216,19 +1231,19 @@
         <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G27" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H27" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1236,19 +1251,19 @@
         <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G28" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H28" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1256,19 +1271,19 @@
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C29" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G29" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H29" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1276,19 +1291,19 @@
         <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G30" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1296,19 +1311,19 @@
         <v>37</v>
       </c>
       <c r="B31" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G31" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H31" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1316,19 +1331,19 @@
         <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G32" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H32" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1336,19 +1351,19 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C33" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G33" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H33" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1356,19 +1371,19 @@
         <v>40</v>
       </c>
       <c r="B34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C34" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G34" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H34" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1376,19 +1391,19 @@
         <v>41</v>
       </c>
       <c r="B35" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C35" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G35" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H35" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1396,19 +1411,19 @@
         <v>42</v>
       </c>
       <c r="B36" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C36" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G36" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H36" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1416,19 +1431,19 @@
         <v>43</v>
       </c>
       <c r="B37" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G37" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H37" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1436,19 +1451,19 @@
         <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C38" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G38" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H38" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -1456,19 +1471,19 @@
         <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C39" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G39" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H39" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -1476,19 +1491,19 @@
         <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C40" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G40" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H40" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -1496,19 +1511,19 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C41" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G41" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H41" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -1516,19 +1531,19 @@
         <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C42" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G42" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H42" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -1536,19 +1551,19 @@
         <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C43" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G43" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H43" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -1556,19 +1571,19 @@
         <v>50</v>
       </c>
       <c r="B44" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C44" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G44" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H44" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -1576,19 +1591,19 @@
         <v>51</v>
       </c>
       <c r="B45" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C45" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G45" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H45" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -1596,19 +1611,19 @@
         <v>52</v>
       </c>
       <c r="B46" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C46" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G46" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H46" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -1616,19 +1631,19 @@
         <v>53</v>
       </c>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C47" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G47" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H47" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -1636,19 +1651,19 @@
         <v>54</v>
       </c>
       <c r="B48" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C48" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G48" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H48" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -1656,19 +1671,59 @@
         <v>55</v>
       </c>
       <c r="B49" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" t="s">
+        <v>59</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G49" t="s">
+        <v>111</v>
+      </c>
+      <c r="H49" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" t="s">
         <v>56</v>
       </c>
-      <c r="C49" t="s">
+      <c r="B50" t="s">
+        <v>58</v>
+      </c>
+      <c r="C50" t="s">
+        <v>59</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G50" t="s">
+        <v>111</v>
+      </c>
+      <c r="H50" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
         <v>57</v>
       </c>
-      <c r="F49" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G49" t="s">
-        <v>106</v>
-      </c>
-      <c r="H49" t="s">
-        <v>107</v>
+      <c r="B51" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" t="s">
+        <v>59</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="G51" t="s">
+        <v>111</v>
+      </c>
+      <c r="H51" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1721,6 +1776,8 @@
     <hyperlink ref="F47" r:id="rId46"/>
     <hyperlink ref="F48" r:id="rId47"/>
     <hyperlink ref="F49" r:id="rId48"/>
+    <hyperlink ref="F50" r:id="rId49"/>
+    <hyperlink ref="F51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>